<commit_message>
Cap nhat tai lieu SRS va Product Backlog sang kien truc Non-MVC (Razor Pages MVVM + Minimal Web API)
</commit_message>
<xml_diff>
--- a/docs/Product_Backlog_EcoBike.xlsx
+++ b/docs/Product_Backlog_EcoBike.xlsx
@@ -170,7 +170,7 @@
       </c>
       <c r="C2" s="0" t="inlineStr">
         <is>
-          <t>Khởi tạo kiến trúc ASP.NET Core 9 MVC</t>
+          <t>Khởi tạo kiến trúc ASP.NET Core 9 Razor Pages (MVVM) + 3-Layer Services</t>
         </is>
       </c>
       <c r="D2" s="0" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t>Dashboard Quản trị sàn (AdminController)</t>
+          <t>Dashboard Quản trị sàn (Pages/Admin (AdminDashboardViewModel))</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">

</xml_diff>